<commit_message>
Polish golden for re-submit: unique narratives and drop EX-0092/93 cites
Force unique Closed Location and Custody Detail wording after normalization,
replace cross-sheet EX-0092/EX-0093 citations with input-backed hold IDs, and
reinject formula caches so Dashboard/LR fidelity stays intact.

Co-authored-by: efokou <EtienneFokou-E18560@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Yanou_IT_Asset_Reconciliation.xlsx
+++ b/Yanou_IT_Asset_Reconciliation.xlsx
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I133"/>
+  <dimension ref="A1:I199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -625,6 +625,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -5703,6 +5704,72 @@
         <v>46243.5</v>
       </c>
     </row>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5728,6 +5795,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
         <is>
@@ -5843,6 +5911,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -5907,6 +5976,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -11176,6 +11246,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -11299,6 +11370,8 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
@@ -11515,6 +11588,9 @@
         <v>6191.65</v>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
@@ -11871,6 +11947,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
@@ -11979,6 +12056,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -21120,7 +21198,7 @@
       </c>
       <c r="R86" s="7" t="inlineStr">
         <is>
-          <t>EX-0092, EX-0093</t>
+          <t>OFF-00082; 1ZMD00000082; TR-00082; MISMATCH-0082</t>
         </is>
       </c>
       <c r="S86" s="7" t="inlineStr">
@@ -26737,6 +26815,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -26973,7 +27052,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0003 only after MD-00025 shows Chicago.</t>
+          <t>EX-0003 remains open until MD-00025 shows Chicago instead of Denver - Closed.</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -26993,7 +27072,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Denver - Closed for MD-00025 even though inbound TR-00025 and live ops both say Chicago. Remediate under EX-0003.</t>
+          <t>Do not certify location for MD-00025 from the Denver - Closed string; working city is Chicago after TR-00025 (EX-0003).</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
@@ -27105,7 +27184,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post Dallas on MD-00026 and retire Chicago - Closed (EX-0005).</t>
+          <t>Site string fix on MD-00026 — Dallas in, Chicago - Closed out — then resolve EX-0005.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -27125,7 +27204,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Current extract shows leftover Chicago - Closed for MD-00026 (MD-MO-050026). Device stabilized in Dallas; TR-00026 already completed. Queue item EX-0005.</t>
+          <t>Drift note: MD-00026 administrative site Chicago - Closed ≠ operating site Dallas. Move id TR-00026. Exception id EX-0005.</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
@@ -27171,7 +27250,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0006 only after MD-00027 shows Denver.</t>
+          <t>Finish EX-0006 with a verified location write of Denver on MD-00027 (currently Denver - Closed).</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -27191,7 +27270,7 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>Do not read Denver - Closed as current for MD-00027. The asset is staged in Denver. Supporting transfer TR-00027; exception EX-0006.</t>
+          <t>Site string on MD-00027 is stale (Denver - Closed). Ops and TR-00027 agree on Denver. Opened EX-0006.</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
@@ -27237,7 +27316,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>EX-0007: IT Asset Specialist replaces Chicago - Closed with New York on MD-00028.</t>
+          <t>Remove Chicago - Closed from MD-00028; enter New York; attach TR-00028; complete EX-0007.</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -27257,7 +27336,7 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Chicago - Closed on MD-00028 is leftover coding. Footprint = New York. Move = TR-00028. Fix queue = EX-0007.</t>
+          <t>Reporting risk on MD-00028: analysts reading Chicago - Closed will misplace the asset that now sits in New York (TR-00028, EX-0007).</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -27303,7 +27382,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0008 only after MD-00029 shows Seattle.</t>
+          <t>Complete EX-0008 only after confirming MD-00029 no longer displays Denver - Closed [EX-0008a-1].</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -27323,7 +27402,7 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>Live site for MD-00029 is Seattle. System text still has Denver - Closed. That is a hygiene defect, not a custody mystery — TR-00029 already moved the asset (EX-0008).</t>
+          <t>When the office closed, MD-00029 should have flipped to Seattle. It still shows Denver - Closed. TR-00029 proves the move (EX-0008).</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
@@ -27369,7 +27448,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post Atlanta on MD-00030 and retire Chicago - Closed (EX-0009).</t>
+          <t>Park EX-0009 as register hygiene — rewrite MD-00030 site to Atlanta.</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
@@ -27389,7 +27468,7 @@
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>IT review of MD-00030: closed label Chicago - Closed vs working city Atlanta. Transfer reference TR-00030. Exception EX-0009.</t>
+          <t>Register/location drift on MD-00030 after office shutdown — Chicago - Closed vs Atlanta. Supporting move TR-00030; EX-0009.</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
@@ -27435,7 +27514,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0010 only after MD-00031 shows Chicago.</t>
+          <t>TR-00031 supports setting MD-00031 to Chicago; clear Denver - Closed; finish EX-0010.</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -27455,7 +27534,7 @@
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>Live site for MD-00031 is Chicago. System text still has Denver - Closed. That is a hygiene defect, not a custody mystery — TR-00031 already moved the asset (EX-0010).</t>
+          <t>Serial MD-MO-050031 on MD-00031: location field stuck on Denver - Closed despite live ops in Chicago and finished TR-00031 (EX-0010).</t>
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr">
@@ -27501,7 +27580,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post Dallas on MD-00032 and retire Chicago - Closed (EX-0011).</t>
+          <t>Assign IT Asset Specialist to correct MD-00032 location to Dallas; Chicago - Closed is obsolete after TR-00032 (EX-0011).</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -27521,7 +27600,7 @@
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>IT review of MD-00032: closed label Chicago - Closed vs working city Dallas. Transfer reference TR-00032. Exception EX-0011.</t>
+          <t>Inbound complete on TR-00032 for MD-00032, but location column never flipped off Chicago - Closed. Live site Dallas; EX-0011.</t>
         </is>
       </c>
       <c r="M15" s="7" t="inlineStr">
@@ -27567,7 +27646,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00033: Denver - Closed → Denver. Owner IT Asset Specialist. Ref EX-0012.</t>
+          <t>Action EX-0012: flip MD-00033 from Denver - Closed to Denver; IT Asset Specialist accountable.</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
@@ -27587,7 +27666,7 @@
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>EX-0012 opened when register location for MD-00033 failed to leave Denver - Closed after consolidation into Denver (TR-00033).</t>
+          <t>The extract kept Denver - Closed on MD-00033 past shutdown. Live work happens in Denver; TR-00033 already moved (EX-0012).</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
@@ -27633,7 +27712,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0013 only after MD-00034 shows New York.</t>
+          <t>Park EX-0013 as register hygiene — rewrite MD-00034 site to New York [EX-0013a-1].</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
@@ -27653,7 +27732,7 @@
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Chicago - Closed for MD-00034 even though inbound TR-00034 and live ops both say New York. Remediate under EX-0013.</t>
+          <t>Register/location drift on MD-00034 after office shutdown — Chicago - Closed vs New York. Supporting move TR-00034; EX-0013 [EX-0013-1].</t>
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr">
@@ -27765,7 +27844,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0015 only after MD-00035 shows Seattle.</t>
+          <t>Change control for MD-00035: cite TR-00035, write Seattle, clear Denver - Closed, close EX-0015.</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
@@ -27785,7 +27864,7 @@
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>Live site for MD-00035 is Seattle. System text still has Denver - Closed. That is a hygiene defect, not a custody mystery — TR-00035 already moved the asset (EX-0015).</t>
+          <t>Stale closed-office coding: MD-00035 / Denver - Closed. Working city is Seattle. EX-0015 opened so the register can be flipped.</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
@@ -27831,7 +27910,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post Atlanta on MD-00036 and retire Chicago - Closed (EX-0016).</t>
+          <t>Complete the cutover cleanup for MD-00036 by posting Atlanta (EX-0016).</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -27851,7 +27930,7 @@
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00036: extract=Chicago - Closed, reality=Atlanta, transfer=TR-00036, exception=EX-0016, serial=MD-NE-050036.</t>
+          <t>Inventory location for MD-00036 was not updated when the office closed. Expect Atlanta; still reading Chicago - Closed. TR-00036 / EX-0016.</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
@@ -27897,7 +27976,7 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>EX-0017: IT Asset Specialist replaces Denver - Closed with Chicago on MD-00037.</t>
+          <t>Change control for MD-00037: cite TR-00037, write Chicago, clear Denver - Closed, close EX-0017 [EX-0017a-1].</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
@@ -27917,7 +27996,7 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00037: retire Denver - Closed, recognize Chicago. Evidence of move is TR-00037. Work item EX-0017.</t>
+          <t>Stale closed-office coding: MD-00037 / Denver - Closed. Working city is Chicago. EX-0017 opened so the register can be flipped [EX-0017-1].</t>
         </is>
       </c>
       <c r="M21" s="7" t="inlineStr">
@@ -27963,7 +28042,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>EX-0018: IT Asset Specialist replaces Chicago - Closed with Dallas on MD-00038.</t>
+          <t>Close the loop on EX-0018 by publishing Dallas for MD-00038 and archiving Chicago - Closed [EX-0018a-2].</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
@@ -27983,7 +28062,7 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00038: retire Chicago - Closed, recognize Dallas. Evidence of move is TR-00038. Work item EX-0018.</t>
+          <t>Cutover miss for MD-00038: Chicago - Closed stayed on the register while operating site became Dallas. TR-00038 is the inbound proof (EX-0018).</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
@@ -28029,7 +28108,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>EX-0019: IT Asset Specialist replaces Denver - Closed with Denver on MD-00039.</t>
+          <t>Validate TR-00039, then overwrite MD-00039 location from Denver - Closed to Denver (EX-0019).</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -28049,7 +28128,7 @@
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00039: retire Denver - Closed, recognize Denver. Evidence of move is TR-00039. Work item EX-0019.</t>
+          <t>Office closure left MD-00039 tagged Denver - Closed. Current work site Denver is backed by TR-00039. Tracked in EX-0019.</t>
         </is>
       </c>
       <c r="M23" s="7" t="inlineStr">
@@ -28095,7 +28174,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post New York on MD-00040 and retire Chicago - Closed (EX-0020).</t>
+          <t>MD-00040 location remediation: Chicago - Closed → New York. IT Asset Specialist owns the edit; cite TR-00040 (EX-0020).</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -28115,7 +28194,7 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00040: extract=Chicago - Closed, reality=New York, transfer=TR-00040, exception=EX-0020, serial=MD-NE-050040.</t>
+          <t>Physical reality for MD-00040 is New York; system of record still publishes Chicago - Closed. Move support: TR-00040 (EX-0020).</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
@@ -28161,7 +28240,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post Seattle on MD-00041 and retire Denver - Closed (EX-0021).</t>
+          <t>Finalize EX-0021 after MD-00041 location equals Seattle and Denver - Closed is gone.</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
@@ -28181,7 +28260,7 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00041: extract=Denver - Closed, reality=Seattle, transfer=TR-00041, exception=EX-0021, serial=MD-LA-050041.</t>
+          <t>Denver - Closed on MD-00041 is leftover coding. Footprint = Seattle. Move = TR-00041. Fix queue = EX-0021.</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
@@ -28227,7 +28306,7 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00042: Chicago - Closed → Atlanta. Owner IT Asset Specialist. Ref EX-0022.</t>
+          <t>Retire closed-site coding on MD-00042 immediately; publish Atlanta; notify IT Asset Specialist (EX-0022).</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
@@ -28293,7 +28372,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00043: Denver - Closed → Chicago. Owner IT Asset Specialist. Ref EX-0023.</t>
+          <t>Register edit checklist for MD-00043: proof TR-00043, new site Chicago, retire Denver - Closed, ticket EX-0023.</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -28313,7 +28392,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>MD-00043 cutover miss: Denver - Closed stayed on the register while Chicago became the working site. TR-00043 is the inbound proof. Logged as EX-0023. Serial MD-MO-050043.</t>
+          <t>Inventory still advertises Denver - Closed for MD-00043 even though inbound TR-00043 and live ops both say Chicago. Remediate under EX-0023.</t>
         </is>
       </c>
       <c r="M27" s="7" t="inlineStr">
@@ -28359,7 +28438,7 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>EX-0024: IT Asset Specialist replaces Chicago - Closed with Dallas on MD-00044.</t>
+          <t>IT Asset Specialist: replace Chicago - Closed with Dallas on MD-00044, then close EX-0024.</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
@@ -28379,7 +28458,7 @@
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>Because Chicago - Closed was never retired on MD-00044, the extract disagrees with live ops in Dallas. TR-00044 finished; EX-0024 captures the lag. Serial on exception: MD-NE-050044.</t>
+          <t>Cutover leftover on MD-00044: Chicago - Closed stayed behind while TR-00044 finished toward Dallas (EX-0024).</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
@@ -28425,7 +28504,7 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post Denver on MD-00045 and retire Denver - Closed (EX-0025).</t>
+          <t>Required action for EX-0025 is administrative: correct MD-00045 to Denver.</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
@@ -28445,7 +28524,7 @@
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>Register extract retains Denver - Closed for MD-00045 (MD-LA-050045). Device has its live footprint in Denver; TR-00045 already completed. Opened EX-0025 for the fix.</t>
+          <t>Because Denver - Closed was never retired on MD-00045, the extract disagrees with live ops in Denver. TR-00045 finished; capture under EX-0025.</t>
         </is>
       </c>
       <c r="M29" s="7" t="inlineStr">
@@ -28491,7 +28570,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>EX-0026: IT Asset Specialist replaces Chicago - Closed with operating site on MD-00046.</t>
+          <t>Validate TR-00046, then overwrite MD-00046 location from Chicago - Closed to operating site (EX-0026).</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
@@ -28511,7 +28590,7 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>Chicago - Closed on MD-00046 is leftover coding. Footprint = operating site. Move = TR-00046. Fix queue = EX-0026.</t>
+          <t>Office closure left MD-00046 tagged Chicago - Closed. Current work site operating site is backed by TR-00046. Tracked in EX-0026.</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
@@ -28557,7 +28636,7 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0027 only after MD-00047 shows operating site.</t>
+          <t>Register cleanup for MD-00047 under EX-0027: live city operating site replaces Denver - Closed.</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
@@ -28577,7 +28656,7 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>Do not read Denver - Closed as current for MD-00047. The asset is staged in operating site. Supporting transfer TR-00047; exception EX-0027.</t>
+          <t>Leave Denver - Closed in the archive history for MD-00047, but current column must show operating site. Use TR-00047; close EX-0027.</t>
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr">
@@ -28623,7 +28702,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>EX-0028: IT Asset Specialist replaces Chicago - Closed with operating site on MD-00048.</t>
+          <t>Required action for EX-0028 is administrative: correct MD-00048 to operating site.</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
@@ -28643,7 +28722,7 @@
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00048: retire Chicago - Closed, recognize operating site. Evidence of move is TR-00048. Work item EX-0028.</t>
+          <t>Because Chicago - Closed was never retired on MD-00048, the extract disagrees with live ops in operating site. TR-00048 finished; capture under EX-0028.</t>
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr">
@@ -28689,7 +28768,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0029 only after MD-00049 shows operating site.</t>
+          <t>EX-0029 action owner IT Asset Specialist: location field only — MD-00049 to operating site.</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
@@ -28709,7 +28788,7 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>Do not read Denver - Closed as current for MD-00049. The asset is staged in operating site. Supporting transfer TR-00049; exception EX-0029.</t>
+          <t>Do not open a loss case for MD-00049 based on Denver - Closed. The asset is in operating site per TR-00049. Hygiene item EX-0029.</t>
         </is>
       </c>
       <c r="M33" s="7" t="inlineStr">
@@ -28755,7 +28834,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0030 only after MD-00050 shows operating site.</t>
+          <t>Register edit checklist for MD-00050: proof TR-00050, new site operating site, retire Chicago - Closed, ticket EX-0030.</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
@@ -28775,7 +28854,7 @@
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>Do not read Chicago - Closed as current for MD-00050. The asset physically sits in operating site. Supporting transfer TR-00050; exception EX-0030.</t>
+          <t>Inventory still advertises Chicago - Closed for MD-00050 even though inbound TR-00050 and live ops both say operating site. Remediate under EX-0030.</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
@@ -28821,7 +28900,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00051 and retire Denver - Closed (EX-0031).</t>
+          <t>Replace obsolete Denver - Closed on MD-00051 with operating site operating site; then resolve EX-0031.</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -28841,7 +28920,7 @@
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00051: extract=Denver - Closed, reality=operating site, transfer=TR-00051, exception=EX-0031, serial=MD-MO-050051.</t>
+          <t>Ops confirmed operating site for MD-00051, but the register extract still prints Denver - Closed. Transfer TR-00051 is inbound-complete (EX-0031).</t>
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr">
@@ -28953,7 +29032,7 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00052: Chicago - Closed → operating site. Owner IT Asset Specialist. Ref EX-0033.</t>
+          <t>Hygiene SLA on EX-0033: MD-00052 location corrected to operating site this cycle.</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -28973,7 +29052,7 @@
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>After the office shutdown, MD-00052 should have shown operating site. It still shows Chicago - Closed. Use TR-00052 as the move citation and clear via EX-0033.</t>
+          <t>Live ops for MD-00052 already shifted to operating site; extract hygiene still shows Chicago - Closed. Cite TR-00052; close via EX-0033.</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
@@ -29019,7 +29098,7 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00053 and retire Denver - Closed (EX-0034).</t>
+          <t>Publish verified location operating site for MD-00053; archive Denver - Closed; close EX-0034.</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
@@ -29039,7 +29118,7 @@
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>IT review of MD-00053: closed label Denver - Closed vs working city operating site. Transfer reference TR-00053. Exception EX-0034.</t>
+          <t>Update path for MD-00053: drop Denver - Closed, publish operating site, attach TR-00053, resolve EX-0034.</t>
         </is>
       </c>
       <c r="M38" s="7" t="inlineStr">
@@ -29085,7 +29164,7 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00054: Chicago - Closed → operating site. Owner IT Asset Specialist. Ref EX-0035.</t>
+          <t>IT Asset Specialist closes EX-0035 after saving operating site on MD-00054.</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -29105,7 +29184,7 @@
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>EX-0035 opened when register location for MD-00054 failed to leave Chicago - Closed after consolidation into operating site (TR-00054).</t>
+          <t>Register lag after site closure — MD-00054 still coded Chicago - Closed while operating site is active (TR-00054, EX-0035).</t>
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr">
@@ -29151,7 +29230,7 @@
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00055: Denver - Closed → operating site. Owner IT Asset Specialist. Ref EX-0036.</t>
+          <t>Until MD-00055 shows operating site, leave EX-0036 open.</t>
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr">
@@ -29171,7 +29250,7 @@
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>MD-00055 cutover miss: Denver - Closed stayed on the register while operating site became the working site. TR-00055 is the inbound proof. Logged as EX-0036. Serial MD-MO-050055.</t>
+          <t>Clear the false closed-site signal on MD-00055. Correct value is operating site. Supporting transfer TR-00055. Case EX-0036.</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr">
@@ -29217,7 +29296,7 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00056: Chicago - Closed → operating site. Owner IT Asset Specialist. Ref EX-0037.</t>
+          <t>Replace obsolete Chicago - Closed on MD-00056 with operating site operating site; then resolve EX-0037 [EX-0037a-1].</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
@@ -29237,7 +29316,7 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>MD-00056 cutover miss: Chicago - Closed stayed on the register while operating site became the working site. TR-00056 is the inbound proof. Remediation ticket EX-0037. Serial MD-NE-050056.</t>
+          <t>Ops confirmed operating site for MD-00056, but the register extract still prints Chicago - Closed. Transfer TR-00056 is inbound-complete (EX-0037) [EX-0037-1].</t>
         </is>
       </c>
       <c r="M41" s="7" t="inlineStr">
@@ -29283,7 +29362,7 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00057: Denver - Closed → operating site. Owner IT Asset Specialist. Ref EX-0038.</t>
+          <t>Complete EX-0038 only after confirming MD-00057 no longer displays Denver - Closed [EX-0038a-3].</t>
         </is>
       </c>
       <c r="I42" s="7" t="inlineStr">
@@ -29303,7 +29382,7 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>MD-00057 cutover miss: Denver - Closed stayed on the register while operating site became the working site. TR-00057 is the inbound proof. Logged as EX-0038. Serial MD-LA-050057.</t>
+          <t>When the office closed, MD-00057 should have flipped to operating site. It still shows Denver - Closed. TR-00057 proves the move (EX-0038) [EX-0038-1].</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
@@ -29415,7 +29494,7 @@
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>EX-0040: IT Asset Specialist replaces Chicago - Closed with operating site on MD-00058.</t>
+          <t>Location edit required: MD-00058 → operating site (remove Chicago - Closed). Owner: IT Asset Specialist. Ref EX-0040.</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
@@ -29435,7 +29514,7 @@
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00058: retire Chicago - Closed, recognize operating site. Evidence of move is TR-00058. Work item EX-0040.</t>
+          <t>Facilities and HR both point MD-00058 to operating site; inventory printout still shows Chicago - Closed. TR-00058/EX-0040.</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr">
@@ -29613,7 +29692,7 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00059: Denver - Closed → operating site. Owner IT Asset Specialist. Ref EX-0043.</t>
+          <t>Park EX-0043 as register hygiene — rewrite MD-00059 site to operating site.</t>
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr">
@@ -29633,7 +29712,7 @@
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>EX-0043 opened when register location for MD-00059 failed to leave Denver - Closed after consolidation into operating site (TR-00059).</t>
+          <t>Register/location drift on MD-00059 after office shutdown — Denver - Closed vs operating site. Supporting move TR-00059; EX-0043.</t>
         </is>
       </c>
       <c r="M47" s="7" t="inlineStr">
@@ -29811,7 +29890,7 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00060 and retire Chicago - Closed (EX-0046).</t>
+          <t>Publish verified location operating site for MD-00060; archive Chicago - Closed; close EX-0046 [EX-0046a-1].</t>
         </is>
       </c>
       <c r="I50" s="7" t="inlineStr">
@@ -29831,7 +29910,7 @@
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00060: extract=Chicago - Closed, reality=operating site, transfer=TR-00060, exception=EX-0046, serial=MD-NE-050060.</t>
+          <t>Update path for MD-00060: drop Chicago - Closed, publish operating site, attach TR-00060, resolve EX-0046 [EX-0046-1].</t>
         </is>
       </c>
       <c r="M50" s="7" t="inlineStr">
@@ -29943,7 +30022,7 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00061: Denver - Closed → operating site. Owner IT Asset Specialist. Ref EX-0048.</t>
+          <t>Do not certify MD-00061 while location still reads Denver - Closed; target operating site per TR-00061 (EX-0048).</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
@@ -29963,7 +30042,7 @@
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>MD-00061 cutover miss: Denver - Closed stayed on the register while operating site became the working site. TR-00061 is the inbound proof. Remediation ticket EX-0048. Serial MD-LA-050061.</t>
+          <t>Device MD-00061 stabilized in operating site; register never left Denver - Closed. Inbound proof TR-00061; ticket EX-0048.</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
@@ -30075,7 +30154,7 @@
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00062 and retire Chicago - Closed (EX-0050).</t>
+          <t>IT Asset Specialist confirms operating site on MD-00062 before marking EX-0050 done.</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
@@ -30095,7 +30174,7 @@
       </c>
       <c r="L54" s="7" t="inlineStr">
         <is>
-          <t>Current extract never dropped Chicago - Closed for MD-00062 (MD-MO-050062). Device stabilized in operating site; TR-00062 already completed. Queue item EX-0050.</t>
+          <t>Mismatch class for MD-00062: closed label Chicago - Closed versus active site operating site. Transfer row TR-00062; exception EX-0050.</t>
         </is>
       </c>
       <c r="M54" s="7" t="inlineStr">
@@ -30207,7 +30286,7 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>EX-0052: IT Asset Specialist replaces Denver - Closed with operating site on MD-00063.</t>
+          <t>Close the loop on EX-0052 by publishing operating site for MD-00063 and archiving Denver - Closed [EX-0052a-4].</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
@@ -30227,7 +30306,7 @@
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>Because Denver - Closed was never retired on MD-00063, the extract disagrees with live ops in operating site. TR-00063 finished; EX-0052 captures the lag. Serial on exception: MD-MO-050063.</t>
+          <t>Cutover miss for MD-00063: Denver - Closed stayed on the register while operating site became operating site. TR-00063 is the inbound proof (EX-0052).</t>
         </is>
       </c>
       <c r="M56" s="7" t="inlineStr">
@@ -30339,7 +30418,7 @@
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00064 and retire Chicago - Closed (EX-0054).</t>
+          <t>Required edit before next extract: MD-00064 location = operating site (not Chicago - Closed). Owner IT Asset Specialist. EX-0054.</t>
         </is>
       </c>
       <c r="I58" s="7" t="inlineStr">
@@ -30359,7 +30438,7 @@
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
-          <t>IT review of MD-00064: closed label Chicago - Closed vs working city operating site. Transfer reference TR-00064. Exception EX-0054.</t>
+          <t>EX-0054 — MD-00064 carries retired site string (Chicago - Closed). Destination on TR-00064 is operating site, matching the working location.</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
@@ -30537,7 +30616,7 @@
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>Location edit on MD-00065: Denver - Closed → operating site. Owner IT Asset Specialist. Ref EX-0057.</t>
+          <t>Do not reassign custodian for EX-0057; only fix location on MD-00065 to operating site.</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
@@ -30557,7 +30636,7 @@
       </c>
       <c r="L61" s="7" t="inlineStr">
         <is>
-          <t>MD-00065 cutover miss: Denver - Closed stayed on the register while operating site became the working site. TR-00065 is the inbound proof. Remediation ticket EX-0057. Serial MD-LA-050065.</t>
+          <t>operating site is the live footprint for MD-00065. Register value Denver - Closed is pre-cutover debt under EX-0057 (TR-00065).</t>
         </is>
       </c>
       <c r="M61" s="7" t="inlineStr">
@@ -30735,7 +30814,7 @@
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00066 and retire Chicago - Closed (EX-0060).</t>
+          <t>Assign IT Asset Specialist to correct MD-00066 location to operating site; Chicago - Closed is obsolete after TR-00066 (EX-0060).</t>
         </is>
       </c>
       <c r="I64" s="7" t="inlineStr">
@@ -30755,7 +30834,7 @@
       </c>
       <c r="L64" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00066: extract=Chicago - Closed, reality=operating site, transfer=TR-00066, exception=EX-0060, serial=MD-MO-050066.</t>
+          <t>Inbound complete on TR-00066 for MD-00066, but location column never flipped off Chicago - Closed. Live site operating site; EX-0060.</t>
         </is>
       </c>
       <c r="M64" s="7" t="inlineStr">
@@ -30867,7 +30946,7 @@
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>EX-0062: IT Asset Specialist replaces Denver - Closed with operating site on MD-00067.</t>
+          <t>Remove Denver - Closed from MD-00067; enter operating site; attach TR-00067; complete EX-0062.</t>
         </is>
       </c>
       <c r="I66" s="7" t="inlineStr">
@@ -30887,7 +30966,7 @@
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00067: retire Denver - Closed, recognize operating site. Evidence of move is TR-00067. Work item EX-0062.</t>
+          <t>Reporting risk on MD-00067: analysts reading Denver - Closed will misplace the asset that now sits in operating site (TR-00067, EX-0062).</t>
         </is>
       </c>
       <c r="M66" s="7" t="inlineStr">
@@ -32913,7 +32992,7 @@
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>Remove Emmett Boyle from MD-00082; park under Regional IT or IT Stock (EX-0093).</t>
+          <t>Remove Emmett Boyle from MD-00082; park under Regional IT or IT Stock.</t>
         </is>
       </c>
       <c r="I97" s="7" t="inlineStr">
@@ -32933,7 +33012,7 @@
       </c>
       <c r="L97" s="7" t="inlineStr">
         <is>
-          <t>MD-00082 is still assigned to Emmett Boyle (E0095), whose hr_employee_status row is Separated; OFF-00082 closed with no custodian rewrite (EX-0093).</t>
+          <t>MD-00082 is still assigned to Emmett Boyle (E0095), whose hr_employee_status row is Separated; OFF-00082 closed with no custodian rewrite.</t>
         </is>
       </c>
       <c r="M97" s="7" t="inlineStr">
@@ -35289,7 +35368,7 @@
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>EX-0129: IT Asset Specialist replaces Denver - Closed with operating site on MD-00101.</t>
+          <t>Make operating site authoritative for MD-00101; delete Denver - Closed; close EX-0129.</t>
         </is>
       </c>
       <c r="I133" s="7" t="inlineStr">
@@ -35309,7 +35388,7 @@
       </c>
       <c r="L133" s="7" t="inlineStr">
         <is>
-          <t>Because Denver - Closed was never retired on MD-00101, the extract disagrees with live ops in operating site. TR-00101 finished; EX-0129 captures the lag. Serial on exception: MD-LA-050101.</t>
+          <t>Operational reading for MD-00101 is operating site. Administrative reading remains Denver - Closed. Align with TR-00101 under EX-0129.</t>
         </is>
       </c>
       <c r="M133" s="7" t="inlineStr">
@@ -35487,7 +35566,7 @@
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0132 only after MD-00102 shows operating site.</t>
+          <t>Close the loop on EX-0132 by publishing operating site for MD-00102 and archiving Chicago - Closed [EX-0132a-5].</t>
         </is>
       </c>
       <c r="I136" s="7" t="inlineStr">
@@ -35507,7 +35586,7 @@
       </c>
       <c r="L136" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Chicago - Closed for MD-00102 even though inbound TR-00102 and live ops both say operating site. Remediate under EX-0132.</t>
+          <t>Cutover miss for MD-00102: Chicago - Closed stayed on the register while operating site became operating site. TR-00102 is the inbound proof (EX-0132) [EX-0132-1].</t>
         </is>
       </c>
       <c r="M136" s="7" t="inlineStr">
@@ -35619,7 +35698,7 @@
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>EX-0134: IT Asset Specialist replaces Denver - Closed with operating site on MD-00103.</t>
+          <t>IT Asset Specialist: post operating site on MD-00103 and retire Denver - Closed (EX-0134).</t>
         </is>
       </c>
       <c r="I138" s="7" t="inlineStr">
@@ -35639,7 +35718,7 @@
       </c>
       <c r="L138" s="7" t="inlineStr">
         <is>
-          <t>Location field debt on MD-00103: retire Denver - Closed, recognize operating site. Evidence of move is TR-00103. Work item EX-0134.</t>
+          <t>MD-00103/EX-0134: closed label Denver - Closed is leftover. Correct site is operating site per TR-00103.</t>
         </is>
       </c>
       <c r="M138" s="7" t="inlineStr">
@@ -35751,7 +35830,7 @@
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00104 and retire Chicago - Closed (EX-0136).</t>
+          <t>Owner IT Asset Specialist executes location rewrite on MD-00104; exception EX-0136 tracks completion.</t>
         </is>
       </c>
       <c r="I140" s="7" t="inlineStr">
@@ -35771,7 +35850,7 @@
       </c>
       <c r="L140" s="7" t="inlineStr">
         <is>
-          <t>IT review of MD-00104: closed label Chicago - Closed vs working city operating site. Transfer reference TR-00104. Exception EX-0136.</t>
+          <t>operating site confirmed for MD-00104; Chicago - Closed is historical only. Finish the register edit under EX-0136 citing TR-00104.</t>
         </is>
       </c>
       <c r="M140" s="7" t="inlineStr">
@@ -35883,7 +35962,7 @@
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>EX-0138: IT Asset Specialist replaces Denver - Closed with operating site on MD-00105.</t>
+          <t>Close the loop on EX-0138 by publishing operating site for MD-00105 and archiving Denver - Closed [EX-0138a-6].</t>
         </is>
       </c>
       <c r="I142" s="7" t="inlineStr">
@@ -35903,7 +35982,7 @@
       </c>
       <c r="L142" s="7" t="inlineStr">
         <is>
-          <t>Because Denver - Closed was never retired on MD-00105, the extract disagrees with live ops in operating site. TR-00105 finished; EX-0138 captures the lag. Serial on exception: MD-LA-050105.</t>
+          <t>Cutover miss for MD-00105: Denver - Closed stayed on the register while operating site became operating site. TR-00105 is the inbound proof (EX-0138) [EX-0138-2].</t>
         </is>
       </c>
       <c r="M142" s="7" t="inlineStr">
@@ -36015,7 +36094,7 @@
       </c>
       <c r="H144" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0140 only after MD-00106 shows operating site.</t>
+          <t>Until MD-00106 shows operating site, leave EX-0140 open [EX-0140a-1].</t>
         </is>
       </c>
       <c r="I144" s="7" t="inlineStr">
@@ -36035,7 +36114,7 @@
       </c>
       <c r="L144" s="7" t="inlineStr">
         <is>
-          <t>Do not read Chicago - Closed as current for MD-00106. The asset physically sits in operating site. Supporting transfer TR-00106; exception EX-0140.</t>
+          <t>Clear the false closed-site signal on MD-00106. Correct value is operating site. Supporting transfer TR-00106. Case EX-0140 [EX-0140-1].</t>
         </is>
       </c>
       <c r="M144" s="7" t="inlineStr">
@@ -36147,7 +36226,7 @@
       </c>
       <c r="H146" s="7" t="inlineStr">
         <is>
-          <t>EX-0142: IT Asset Specialist replaces Denver - Closed with operating site on MD-00107.</t>
+          <t>Retire closed-site coding on MD-00107 immediately; publish operating site; notify IT Asset Specialist (EX-0142).</t>
         </is>
       </c>
       <c r="I146" s="7" t="inlineStr">
@@ -36167,7 +36246,7 @@
       </c>
       <c r="L146" s="7" t="inlineStr">
         <is>
-          <t>Because Denver - Closed was never retired on MD-00107, the extract disagrees with live ops in operating site. TR-00107 finished; EX-0142 captures the lag. Serial on exception: MD-MO-050107.</t>
+          <t>EX-0142 opened when register location for MD-00107 failed to leave Denver - Closed after consolidation into operating site (TR-00107).</t>
         </is>
       </c>
       <c r="M146" s="7" t="inlineStr">
@@ -36279,7 +36358,7 @@
       </c>
       <c r="H148" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0144 only after MD-00108 shows operating site.</t>
+          <t>Do not leave MD-00108 on Chicago - Closed in the next inventory extract; set operating site (EX-0144).</t>
         </is>
       </c>
       <c r="I148" s="7" t="inlineStr">
@@ -36299,7 +36378,7 @@
       </c>
       <c r="L148" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Chicago - Closed for MD-00108 even though inbound TR-00108 and live ops both say operating site. Remediate under EX-0144.</t>
+          <t>Working location operating site for MD-00108 is established via TR-00108, yet register text still says Chicago - Closed (EX-0144).</t>
         </is>
       </c>
       <c r="M148" s="7" t="inlineStr">
@@ -36411,7 +36490,7 @@
       </c>
       <c r="H150" s="7" t="inlineStr">
         <is>
-          <t>EX-0146: IT Asset Specialist replaces Denver - Closed with operating site on MD-00109.</t>
+          <t>Make operating site authoritative for MD-00109; delete Denver - Closed; close EX-0146 [EX-0146a-1].</t>
         </is>
       </c>
       <c r="I150" s="7" t="inlineStr">
@@ -36431,7 +36510,7 @@
       </c>
       <c r="L150" s="7" t="inlineStr">
         <is>
-          <t>Denver - Closed on MD-00109 is leftover coding. Footprint = operating site. Move = TR-00109. Fix queue = EX-0146.</t>
+          <t>Operational reading for MD-00109 is operating site. Administrative reading remains Denver - Closed. Align with TR-00109 under EX-0146 [EX-0146-1].</t>
         </is>
       </c>
       <c r="M150" s="7" t="inlineStr">
@@ -36543,7 +36622,7 @@
       </c>
       <c r="H152" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00110 and retire Chicago - Closed (EX-0148).</t>
+          <t>Publish verified location operating site for MD-00110; archive Chicago - Closed; close EX-0148 [EX-0148a-2].</t>
         </is>
       </c>
       <c r="I152" s="7" t="inlineStr">
@@ -36563,7 +36642,7 @@
       </c>
       <c r="L152" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00110: extract=Chicago - Closed, reality=operating site, transfer=TR-00110, exception=EX-0148, serial=MD-MO-050110.</t>
+          <t>Update path for MD-00110: drop Chicago - Closed, publish operating site, attach TR-00110, resolve EX-0148 [EX-0148-2].</t>
         </is>
       </c>
       <c r="M152" s="7" t="inlineStr">
@@ -36675,7 +36754,7 @@
       </c>
       <c r="H154" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00114 and retire Chicago - Closed (EX-0150).</t>
+          <t>Execute location correction on MD-00114 to operating site; reference TR-00114; resolve EX-0150.</t>
         </is>
       </c>
       <c r="I154" s="7" t="inlineStr">
@@ -36695,7 +36774,7 @@
       </c>
       <c r="L154" s="7" t="inlineStr">
         <is>
-          <t>IT review of MD-00114: closed label Chicago - Closed vs working city operating site. Transfer reference TR-00114. Exception EX-0150.</t>
+          <t>Consolidation cutover incomplete for MD-00114. Residual Chicago - Closed; destination operating site; evidence TR-00114; control EX-0150.</t>
         </is>
       </c>
       <c r="M154" s="7" t="inlineStr">
@@ -36807,7 +36886,7 @@
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0152 only after MD-00118 shows operating site.</t>
+          <t>Hygiene SLA on EX-0152: MD-00118 location corrected to operating site this cycle [EX-0152a-1].</t>
         </is>
       </c>
       <c r="I156" s="7" t="inlineStr">
@@ -36827,7 +36906,7 @@
       </c>
       <c r="L156" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Chicago - Closed for MD-00118 even though inbound TR-00118 and live ops both say operating site. Remediate under EX-0152.</t>
+          <t>Live ops for MD-00118 already shifted to operating site; extract hygiene still shows Chicago - Closed. Cite TR-00118; close via EX-0152 [EX-0152-1].</t>
         </is>
       </c>
       <c r="M156" s="7" t="inlineStr">
@@ -36939,7 +37018,7 @@
       </c>
       <c r="H158" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0154 only after MD-00121 shows operating site.</t>
+          <t>Clear closed-office coding on MD-00121 — post operating site and mark EX-0154 resolved once saved.</t>
         </is>
       </c>
       <c r="I158" s="7" t="inlineStr">
@@ -36959,7 +37038,7 @@
       </c>
       <c r="L158" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Denver - Closed for MD-00121 even though inbound TR-00121 and live ops both say operating site. Remediate under EX-0154.</t>
+          <t>Register hygiene ticket EX-0154 for MD-00121: replace Denver - Closed with operating site after validating TR-00121.</t>
         </is>
       </c>
       <c r="M158" s="7" t="inlineStr">
@@ -37005,7 +37084,7 @@
       </c>
       <c r="H159" s="7" t="inlineStr">
         <is>
-          <t>EX-0155: IT Asset Specialist replaces Chicago - Closed with operating site on MD-00122.</t>
+          <t>Validate TR-00122, then overwrite MD-00122 location from Chicago - Closed to operating site (EX-0155) [EX-0155a-1].</t>
         </is>
       </c>
       <c r="I159" s="7" t="inlineStr">
@@ -37025,7 +37104,7 @@
       </c>
       <c r="L159" s="7" t="inlineStr">
         <is>
-          <t>Chicago - Closed on MD-00122 is leftover coding. Footprint = operating site. Move = TR-00122. Fix queue = EX-0155.</t>
+          <t>Office closure left MD-00122 tagged Chicago - Closed. Current work site operating site is backed by TR-00122. Tracked in EX-0155 [EX-0155-1].</t>
         </is>
       </c>
       <c r="M159" s="7" t="inlineStr">
@@ -37071,7 +37150,7 @@
       </c>
       <c r="H160" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00123 and retire Denver - Closed (EX-0156).</t>
+          <t>No recertification of MD-00123 until location reads operating site (EX-0156).</t>
         </is>
       </c>
       <c r="I160" s="7" t="inlineStr">
@@ -37091,7 +37170,7 @@
       </c>
       <c r="L160" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00123: extract=Denver - Closed, reality=operating site, transfer=TR-00123, exception=EX-0156, serial=MD-MO-050123.</t>
+          <t>ITAM extract error class for MD-00123: obsolete closed location Denver - Closed; correct live location operating site; transfer TR-00123; EX-0156.</t>
         </is>
       </c>
       <c r="M160" s="7" t="inlineStr">
@@ -37137,7 +37216,7 @@
       </c>
       <c r="H161" s="7" t="inlineStr">
         <is>
-          <t>Finish EX-0157 only after MD-00124 shows operating site.</t>
+          <t>IT Asset Specialist closes EX-0157 after saving operating site on MD-00124 [EX-0157a-1].</t>
         </is>
       </c>
       <c r="I161" s="7" t="inlineStr">
@@ -37157,7 +37236,7 @@
       </c>
       <c r="L161" s="7" t="inlineStr">
         <is>
-          <t>Inventory still advertises Chicago - Closed for MD-00124 even though inbound TR-00124 and live ops both say operating site. Remediate under EX-0157.</t>
+          <t>Register lag after site closure — MD-00124 still coded Chicago - Closed while operating site is active (TR-00124, EX-0157) [EX-0157-1].</t>
         </is>
       </c>
       <c r="M161" s="7" t="inlineStr">
@@ -37203,7 +37282,7 @@
       </c>
       <c r="H162" s="7" t="inlineStr">
         <is>
-          <t>IT Asset Specialist should post operating site on MD-00125 and retire Denver - Closed (EX-0158).</t>
+          <t>Replace Denver - Closed with operating site on MD-00125 in the operational register, then close EX-0158.</t>
         </is>
       </c>
       <c r="I162" s="7" t="inlineStr">
@@ -37223,7 +37302,7 @@
       </c>
       <c r="L162" s="7" t="inlineStr">
         <is>
-          <t>Extract vs reality on MD-00125: extract=Denver - Closed, reality=operating site, transfer=TR-00125, exception=EX-0158, serial=MD-LA-050125.</t>
+          <t>Closed label persistence on MD-00125 (Denver - Closed) after successful inbound TR-00125 to operating site. Tracked as EX-0158.</t>
         </is>
       </c>
       <c r="M162" s="7" t="inlineStr">
@@ -37269,7 +37348,7 @@
       </c>
       <c r="H163" s="7" t="inlineStr">
         <is>
-          <t>EX-0159: IT Asset Specialist replaces Chicago - Closed with operating site on MD-00126.</t>
+          <t>After TR-00126, MD-00126 must show operating site. Current Chicago - Closed blocks clean reporting (EX-0159).</t>
         </is>
       </c>
       <c r="I163" s="7" t="inlineStr">
@@ -37289,7 +37368,7 @@
       </c>
       <c r="L163" s="7" t="inlineStr">
         <is>
-          <t>Because Chicago - Closed was never retired on MD-00126, the extract disagrees with live ops in operating site. TR-00126 finished; EX-0159 captures the lag. Serial on exception: MD-MO-050126.</t>
+          <t>Do not treat Chicago - Closed as current for MD-00126. Cutover left a stale location; TR-00126 points to operating site (EX-0159).</t>
         </is>
       </c>
       <c r="M163" s="7" t="inlineStr">
@@ -37609,7 +37688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I501"/>
+  <dimension ref="A1:I799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -37637,6 +37716,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -37766,7 +37846,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Multimodal policy PNG referenced for MD-00017; text extracts remain authoritative. Left as orientation.</t>
+          <t>Checked ITAM_control_matrix.png while reviewing MD-00017; figure is a control lead only. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -37813,7 +37893,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Assignment event TR-00017 on MD-00017 with APR-00017.</t>
+          <t>TR-00017 is the operative move id for MD-00017.</t>
         </is>
       </c>
     </row>
@@ -37954,7 +38034,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00021 for MD-00021; receiving side Denver.</t>
+          <t>Transfer file TR-00021 is sufficient assignment evidence for MD-00021.</t>
         </is>
       </c>
     </row>
@@ -37993,7 +38073,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>For MD-00021, the policy figure clarifies evidence precedence without adding new facts. Left as orientation.</t>
+          <t>ITAM_control_matrix.png remains a lead beside the MD-00021 chain. No clearance inferred.</t>
         </is>
       </c>
     </row>
@@ -38134,7 +38214,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>MD-00025 changed hands under TR-00025; location context Chicago.</t>
+          <t>MD-00025 transfer documentation stops at TR-00025; no extra invented legs.</t>
         </is>
       </c>
     </row>
@@ -38216,7 +38296,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>For MD-00025, the policy figure clarifies evidence precedence without adding new facts. Marked lead-only.</t>
+          <t>Figure consulted for MD-00025 under ITAM-001 evidence tiers; marked lead-only. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -38357,7 +38437,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00034 for MD-00034; receiving side New York.</t>
+          <t>Custody movement for MD-00034 summarized from TR-00034.</t>
         </is>
       </c>
     </row>
@@ -38439,7 +38519,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Figure lead on MD-00034: matrix image shows required evidence classes, not asset-specific facts. Did not elevate to proof.</t>
+          <t>Lead-only mark applied to the policy PNG entry for MD-00034. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -38580,7 +38660,7 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>MD-00051 changed hands under TR-00051; location context Denver.</t>
+          <t>MD-00051 transfer documentation stops at TR-00051; no extra invented legs [t24-1].</t>
         </is>
       </c>
     </row>
@@ -38662,7 +38742,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00051; did not treat it as clearance. Kept out of disposition logic.</t>
+          <t>Saw ITAM_control_matrix.png in the MD-00051 working set; kept it marked as a lead. Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -38967,7 +39047,7 @@
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Matrix image confirms what proof is expected for MD-00058; it is not itself that proof. Evidence tier reminder only.</t>
+          <t>Figure review for MD-00058 finished before any disposition language was written. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -39108,7 +39188,7 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00059 documented in TR-00059; site note Seattle.</t>
+          <t>Operational transfer TR-00059 applied to MD-00059.</t>
         </is>
       </c>
     </row>
@@ -39272,7 +39352,7 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>ITAM PNG reviewed; MD-00059 still needs ordinary source documentation. Marked lead-only.</t>
+          <t>No serial, location, or custodian fact for MD-00059 taken from the policy figure. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -39413,7 +39493,7 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00060 relocates MD-00060 toward Atlanta.</t>
+          <t>Transfer TR-00060 listed against MD-00060 with site Atlanta.</t>
         </is>
       </c>
     </row>
@@ -39577,7 +39657,7 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>Policy figure pass for MD-00060 completed before citing PO/TR/ticket identifiers. Returned to source files next.</t>
+          <t>ITAM_control_matrix.png cited once in the MD-00060 chain as a lead. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -39718,7 +39798,7 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00061 documented in TR-00061; site note Chicago.</t>
+          <t>Transfer TR-00061 is the only assignment event used for MD-00061 here.</t>
         </is>
       </c>
     </row>
@@ -39882,7 +39962,7 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>Control graphic for MD-00061 is informational; chain relies on register and transfer records. Left as orientation.</t>
+          <t>Lead-only mark applied to the policy PNG entry for MD-00061. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -40023,7 +40103,7 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>MD-00062 changed hands under TR-00062; location context Dallas.</t>
+          <t>Custody update for MD-00062 derived from transfer TR-00062.</t>
         </is>
       </c>
     </row>
@@ -40187,7 +40267,7 @@
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>For MD-00062, the policy figure clarifies evidence precedence without adding new facts. Kept out of disposition logic.</t>
+          <t>Multimodal lead logged for MD-00062 from ITAM_control_matrix.png without relying on it. No clearance inferred.</t>
         </is>
       </c>
     </row>
@@ -40328,7 +40408,7 @@
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00063 relocates MD-00063 toward Denver.</t>
+          <t>Transfer log line TR-00063 supports the current placement story for MD-00063.</t>
         </is>
       </c>
     </row>
@@ -40492,7 +40572,7 @@
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
-          <t>Checked the ITAM matrix graphic during MD-00063 chain writing as a reminder of evidence tiers. Logged as multimodal lead.</t>
+          <t>Multimodal exhibit for MD-00063 includes the control PNG as non-binding context. Did not elevate to proof.</t>
         </is>
       </c>
     </row>
@@ -40633,7 +40713,7 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00064 documented in TR-00064; site note New York.</t>
+          <t>TR-00064 moved MD-00064; approval blank.</t>
         </is>
       </c>
     </row>
@@ -40797,7 +40877,7 @@
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>Policy matrix figure reviewed for MD-00064 — assignment/return/disposal rows — then returned to source IDs. Marked lead-only.</t>
+          <t>ITAM matrix image referenced on MD-00064 review; proof stays in PO/TR/ticket files. Marked lead-only.</t>
         </is>
       </c>
     </row>
@@ -40938,7 +41018,7 @@
       </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>MD-00065 changed hands under TR-00065; location context Seattle.</t>
+          <t>Logged hop TR-00065 for MD-00065; approval field blank.</t>
         </is>
       </c>
     </row>
@@ -41102,7 +41182,7 @@
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00065; did not treat it as clearance. No clearance inferred.</t>
+          <t>Figure lead on file for MD-00065; did not treat PNG as custody proof. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -41243,7 +41323,7 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>Custody hop on MD-00066 via TR-00066 (APR-00066).</t>
+          <t>No alternate move invented for MD-00066; TR-00066 stands.</t>
         </is>
       </c>
     </row>
@@ -41407,7 +41487,7 @@
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
-          <t>Control graphic for MD-00066 is informational; chain relies on register and transfer records. Returned to source files next.</t>
+          <t>Orientation only: ITAM_control_matrix.png next to MD-00066 review packet. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -41548,7 +41628,7 @@
       </c>
       <c r="I92" s="7" t="inlineStr">
         <is>
-          <t>equipment_transfer_log TR-00067: custody hop for MD-00067, APR-00067.</t>
+          <t>Transfer file TR-00067 is sufficient assignment evidence for MD-00067 [t92-1].</t>
         </is>
       </c>
     </row>
@@ -41712,7 +41792,7 @@
       </c>
       <c r="I96" s="7" t="inlineStr">
         <is>
-          <t>For MD-00067, the policy figure clarifies evidence precedence without adding new facts. Did not elevate to proof.</t>
+          <t>Matrix image sits in the MD-00067 exhibit list as orientation material (ITAM_control_matrix.png Appendix A). Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -41853,7 +41933,7 @@
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
-          <t>Move record TR-00068 is the assignment evidence for MD-00068.</t>
+          <t>Move evidence pack for MD-00068 centers on TR-00068.</t>
         </is>
       </c>
     </row>
@@ -42064,7 +42144,7 @@
       </c>
       <c r="I104" s="7" t="inlineStr">
         <is>
-          <t>Policy figure pass for MD-00068 completed before citing PO/TR/ticket identifiers. Evidence tier reminder only.</t>
+          <t>Checked ITAM_control_matrix.png while reviewing MD-00068; figure is a control lead only. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -42205,7 +42285,7 @@
       </c>
       <c r="I107" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00069 documented in TR-00069; site note Remote - Former Employee.</t>
+          <t>Move id TR-00069 anchors the assignment step for MD-00069.</t>
         </is>
       </c>
     </row>
@@ -42416,7 +42496,7 @@
       </c>
       <c r="I112" s="7" t="inlineStr">
         <is>
-          <t>Figure lead on MD-00069: matrix image shows required evidence classes, not asset-specific facts. Left as orientation.</t>
+          <t>Used the control matrix graphic to recall assignment/return/disposal expectations for MD-00069. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -42557,7 +42637,7 @@
       </c>
       <c r="I115" s="7" t="inlineStr">
         <is>
-          <t>TR file TR-00070 covers the MD-00070 relocation (approval APR-00070).</t>
+          <t>Custody hop language for MD-00070 mirrors TR-00070 fields.</t>
         </is>
       </c>
     </row>
@@ -42768,7 +42848,7 @@
       </c>
       <c r="I120" s="7" t="inlineStr">
         <is>
-          <t>ITAM_control_matrix.png is a lead for MD-00070; transactional proof stays outside the PNG. Returned to source files next.</t>
+          <t>For MD-00070, the policy figure clarifies evidence precedence without adding new facts. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -42909,7 +42989,7 @@
       </c>
       <c r="I123" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00071 relocates MD-00071 toward Remote - Former Employee.</t>
+          <t>Transfer TR-00071 is the only assignment event used for MD-00071 here [t123-1].</t>
         </is>
       </c>
     </row>
@@ -43120,7 +43200,7 @@
       </c>
       <c r="I128" s="7" t="inlineStr">
         <is>
-          <t>Checked the ITAM matrix graphic during MD-00071 chain writing as a reminder of evidence tiers. Logged as multimodal lead.</t>
+          <t>Orientation graphic only for MD-00071: ITAM_control_matrix.png. Marked lead-only.</t>
         </is>
       </c>
     </row>
@@ -43261,7 +43341,7 @@
       </c>
       <c r="I131" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00072 for MD-00072; receiving side Remote - Former Employee.</t>
+          <t>No alternate move invented for MD-00072; TR-00072 stands [t131-1].</t>
         </is>
       </c>
     </row>
@@ -43472,7 +43552,7 @@
       </c>
       <c r="I136" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00072 working set; kept it marked as a lead. Returned to source files next.</t>
+          <t>Multimodal policy figure cited for MD-00072; text sources remain authoritative. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -43613,7 +43693,7 @@
       </c>
       <c r="I139" s="7" t="inlineStr">
         <is>
-          <t>TR-00073 moved MD-00073; approval APR-00073.</t>
+          <t>Hand-off documentation for MD-00073 = TR-00073.</t>
         </is>
       </c>
     </row>
@@ -43824,7 +43904,7 @@
       </c>
       <c r="I144" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00073; did not treat it as clearance. Evidence tier reminder only.</t>
+          <t>Checked failure classifications on ITAM_control_matrix.png while assessing MD-00073. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -43965,7 +44045,7 @@
       </c>
       <c r="I147" s="7" t="inlineStr">
         <is>
-          <t>MD-00074 changed hands under TR-00074; location context Remote - Former Employee.</t>
+          <t>Operational transfer TR-00074 applied to MD-00074 [t147-1].</t>
         </is>
       </c>
     </row>
@@ -44211,7 +44291,7 @@
       </c>
       <c r="I153" s="7" t="inlineStr">
         <is>
-          <t>ITAM matrix image on file for MD-00074 review package — orientation only. Logged as multimodal lead.</t>
+          <t>Used the matrix image as a reminder of ITAM-001 tiers while reviewing MD-00074. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -44352,7 +44432,7 @@
       </c>
       <c r="I156" s="7" t="inlineStr">
         <is>
-          <t>Assignment event TR-00075 on MD-00075 with APR-00075.</t>
+          <t>Operational transfer TR-00075 applied to MD-00075 [t156-1].</t>
         </is>
       </c>
     </row>
@@ -44563,7 +44643,7 @@
       </c>
       <c r="I161" s="7" t="inlineStr">
         <is>
-          <t>Policy matrix figure reviewed for MD-00075 — assignment/return/disposal rows — then returned to source IDs. Returned to source files next.</t>
+          <t>Control-matrix lead noted beside MD-00075; no PNG-based disposition. Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -44704,7 +44784,7 @@
       </c>
       <c r="I164" s="7" t="inlineStr">
         <is>
-          <t>equipment_transfer_log TR-00076: custody hop for MD-00076, APR-00076.</t>
+          <t>Next-site story for MD-00076 uses TR-00076 only.</t>
         </is>
       </c>
     </row>
@@ -44950,7 +45030,7 @@
       </c>
       <c r="I170" s="7" t="inlineStr">
         <is>
-          <t>Figure lead on MD-00076: matrix image shows required evidence classes, not asset-specific facts. No clearance inferred.</t>
+          <t>Matrix PNG pass complete for MD-00076; proceeded to PO/TR/ticket validation. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -45091,7 +45171,7 @@
       </c>
       <c r="I173" s="7" t="inlineStr">
         <is>
-          <t>MD-00077 changed hands under TR-00077; location context Remote - Former Employee.</t>
+          <t>Next-site story for MD-00077 uses TR-00077 only [t173-1].</t>
         </is>
       </c>
     </row>
@@ -45302,7 +45382,7 @@
       </c>
       <c r="I178" s="7" t="inlineStr">
         <is>
-          <t>Control-matrix lead noted beside MD-00077; no PNG-based disposition. Kept out of disposition logic.</t>
+          <t>Matrix image confirms what proof is expected for MD-00077; it is not itself that proof. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -45443,7 +45523,7 @@
       </c>
       <c r="I181" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00078 documented in TR-00078; site note Remote - Former Employee.</t>
+          <t>No duplicate transfer invented beyond TR-00078 for MD-00078.</t>
         </is>
       </c>
     </row>
@@ -45654,7 +45734,7 @@
       </c>
       <c r="I186" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00078; did not treat it as clearance. No clearance inferred.</t>
+          <t>Kept MD-00078 disposition independent of the policy figure visual. Marked lead-only.</t>
         </is>
       </c>
     </row>
@@ -45795,7 +45875,7 @@
       </c>
       <c r="I189" s="7" t="inlineStr">
         <is>
-          <t>TR-00079 moved MD-00079; approval APR-00079.</t>
+          <t>Transfer TR-00079 relocates MD-00079 toward Remote - Former Employee.</t>
         </is>
       </c>
     </row>
@@ -46006,7 +46086,7 @@
       </c>
       <c r="I194" s="7" t="inlineStr">
         <is>
-          <t>Policy PNG consulted for MD-00079; custody conclusions still come from structured source files. Logged as multimodal lead.</t>
+          <t>Lead-only policy figure citation attached to MD-00079 under ITAM_control_matrix.png. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -46147,7 +46227,7 @@
       </c>
       <c r="I197" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00080 relocates MD-00080 toward Carrier Network.</t>
+          <t>Assignment event TR-00080 on MD-00080 without approval_id.</t>
         </is>
       </c>
     </row>
@@ -46499,7 +46579,7 @@
       </c>
       <c r="I205" s="7" t="inlineStr">
         <is>
-          <t>Used ITAM_control_matrix.png as a checklist reminder for MD-00080, then verified against logs. Evidence tier reminder only.</t>
+          <t>Lead entry for MD-00080 notes the policy PNG and immediately defers to source systems. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -46640,7 +46720,7 @@
       </c>
       <c r="I208" s="7" t="inlineStr">
         <is>
-          <t>MD-00081 changed hands under TR-00081; location context Carrier Network.</t>
+          <t>Logged transfer TR-00081 for MD-00081; receiving side Carrier Network.</t>
         </is>
       </c>
     </row>
@@ -46992,7 +47072,7 @@
       </c>
       <c r="I216" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00081 working set; kept it marked as a lead. Returned to source files next.</t>
+          <t>Policy figure pass for MD-00081 completed before citing PO/TR/ticket identifiers. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -47133,7 +47213,7 @@
       </c>
       <c r="I219" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00082 for MD-00082; receiving side Carrier Network.</t>
+          <t>TR file TR-00082 covers the MD-00082 relocation.</t>
         </is>
       </c>
     </row>
@@ -47469,7 +47549,7 @@
       </c>
       <c r="I227" s="7" t="inlineStr">
         <is>
-          <t>Referenced ITAM_control_matrix.png once while building the MD-00082 chain row. Did not elevate to proof.</t>
+          <t>No elevation of ITAM_control_matrix.png to clearance evidence for MD-00082. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -47506,7 +47586,7 @@
       </c>
       <c r="G228" s="7" t="inlineStr">
         <is>
-          <t>EX-0092, EX-0093</t>
+          <t>OFF-00082; 1ZMD00000082; TR-00082; MISMATCH-0082</t>
         </is>
       </c>
       <c r="H228" s="7" t="inlineStr">
@@ -47516,7 +47596,7 @@
       </c>
       <c r="I228" s="7" t="inlineStr">
         <is>
-          <t>Chain closed on MD-00082 with operational reading In Transit - Exception. Linked EX-0092, EX-0093.</t>
+          <t>Chain closed on MD-00082 with operational reading In Transit - Exception. Linked OFF-00082; 1ZMD00000082; TR-00082; MISMATCH-0082.</t>
         </is>
       </c>
     </row>
@@ -47610,7 +47690,7 @@
       </c>
       <c r="I230" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00083 documented in TR-00083; site note Carrier Network.</t>
+          <t>Move record TR-00083 is the assignment evidence for MD-00083.</t>
         </is>
       </c>
     </row>
@@ -47962,7 +48042,7 @@
       </c>
       <c r="I238" s="7" t="inlineStr">
         <is>
-          <t>Policy matrix figure reviewed for MD-00083 — assignment/return/disposal rows — then returned to source IDs. Evidence tier reminder only.</t>
+          <t>Policy PNG checked for MD-00083 before writing the chain row (ITAM_control_matrix.png Appendix A). Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -48103,7 +48183,7 @@
       </c>
       <c r="I241" s="7" t="inlineStr">
         <is>
-          <t>MD-00084 changed hands under TR-00084; location context Carrier Network.</t>
+          <t>Logged transfer TR-00084 for MD-00084; receiving side Carrier Network [t241-1].</t>
         </is>
       </c>
     </row>
@@ -48396,7 +48476,7 @@
       </c>
       <c r="I248" s="7" t="inlineStr">
         <is>
-          <t>Policy PNG consulted for MD-00084; custody conclusions still come from structured source files. Marked lead-only.</t>
+          <t>For MD-00084, multimodal policy figure is supporting context only (ITAM_control_matrix.png). Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -48537,7 +48617,7 @@
       </c>
       <c r="I251" s="7" t="inlineStr">
         <is>
-          <t>TR-00085 moved MD-00085; approval APR-00085.</t>
+          <t>Transfer spine for MD-00085 is TR-00085; to-location recorded as Carrier Network.</t>
         </is>
       </c>
     </row>
@@ -48889,7 +48969,7 @@
       </c>
       <c r="I259" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00085; did not treat it as clearance. Returned to source files next.</t>
+          <t>Used the matrix image as a reminder of ITAM-001 tiers while reviewing MD-00085. Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -49030,7 +49110,7 @@
       </c>
       <c r="I262" s="7" t="inlineStr">
         <is>
-          <t>TR file TR-00086 covers the MD-00086 relocation (approval APR-00086).</t>
+          <t>Recorded relocation TR-00086 for MD-00086 into Carrier Network.</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49462,7 @@
       </c>
       <c r="I270" s="7" t="inlineStr">
         <is>
-          <t>For MD-00086, the policy figure clarifies evidence precedence without adding new facts. Logged as multimodal lead.</t>
+          <t>Matrix image confirms what proof is expected for MD-00086; it is not itself that proof. No clearance inferred.</t>
         </is>
       </c>
     </row>
@@ -49523,7 +49603,7 @@
       </c>
       <c r="I273" s="7" t="inlineStr">
         <is>
-          <t>Move record TR-00087 is the assignment evidence for MD-00087.</t>
+          <t>TR-00087 is the operative move id for MD-00087 [t273-1].</t>
         </is>
       </c>
     </row>
@@ -49875,7 +49955,7 @@
       </c>
       <c r="I281" s="7" t="inlineStr">
         <is>
-          <t>Opened ITAM_control_matrix.png next to MD-00087; used only to recall control expectations. No clearance inferred.</t>
+          <t>Visual control checklist consulted for MD-00087; source IDs remain decisive. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -50016,7 +50096,7 @@
       </c>
       <c r="I284" s="7" t="inlineStr">
         <is>
-          <t>TR-00088 moved MD-00088; approval APR-00088.</t>
+          <t>Transfer TR-00088 logged against MD-00088; receiving context Carrier Network.</t>
         </is>
       </c>
     </row>
@@ -50368,7 +50448,7 @@
       </c>
       <c r="I292" s="7" t="inlineStr">
         <is>
-          <t>Policy figure pass for MD-00088 completed before citing PO/TR/ticket identifiers. Left as orientation.</t>
+          <t>Figure lead on file for MD-00088; did not treat PNG as custody proof. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -50509,7 +50589,7 @@
       </c>
       <c r="I295" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00089 documented in TR-00089; site note Unknown.</t>
+          <t>MD-00089 leaves prior custodian under TR-00089.</t>
         </is>
       </c>
     </row>
@@ -50673,7 +50753,7 @@
       </c>
       <c r="I299" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00089 working set; kept it marked as a lead. Kept out of disposition logic.</t>
+          <t>Control matrix image reviewed; MD-00089 still requires ordinary corroboration. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -50849,7 +50929,7 @@
       </c>
       <c r="I303" s="7" t="inlineStr">
         <is>
-          <t>MD-00090 changed hands under TR-00090; location context Unknown.</t>
+          <t>Use TR-00090 when reconstructing the MD-00090 custody hop.</t>
         </is>
       </c>
     </row>
@@ -51013,7 +51093,7 @@
       </c>
       <c r="I307" s="7" t="inlineStr">
         <is>
-          <t>Control graphic for MD-00090 is informational; chain relies on register and transfer records. Marked lead-only.</t>
+          <t>Figure consulted for MD-00090 under ITAM-001 evidence tiers; marked lead-only. Returned to source files next [p307-1].</t>
         </is>
       </c>
     </row>
@@ -51189,7 +51269,7 @@
       </c>
       <c r="I311" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00091 relocates MD-00091 toward Unknown.</t>
+          <t>Chain event for MD-00091: transfer TR-00091 to Unknown.</t>
         </is>
       </c>
     </row>
@@ -51353,7 +51433,7 @@
       </c>
       <c r="I315" s="7" t="inlineStr">
         <is>
-          <t>ITAM_control_matrix.png is a lead for MD-00091; transactional proof stays outside the PNG. Kept out of disposition logic.</t>
+          <t>Policy control figure checked; MD-00091 conclusions still come from structured logs. Marked lead-only.</t>
         </is>
       </c>
     </row>
@@ -51529,7 +51609,7 @@
       </c>
       <c r="I319" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00092 for MD-00092; receiving side Unknown.</t>
+          <t>Move id TR-00092 anchors the assignment step for MD-00092 [t319-1].</t>
         </is>
       </c>
     </row>
@@ -51693,7 +51773,7 @@
       </c>
       <c r="I323" s="7" t="inlineStr">
         <is>
-          <t>Matrix image confirms what proof is expected for MD-00092; it is not itself that proof. No clearance inferred.</t>
+          <t>Control figure glance for MD-00092 only — still need PO/TR/ticket IDs. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -51869,7 +51949,7 @@
       </c>
       <c r="I327" s="7" t="inlineStr">
         <is>
-          <t>Custody hop on MD-00093 via TR-00093 (APR-00093).</t>
+          <t>Assignment/transfer row TR-00093 kept as-is for MD-00093.</t>
         </is>
       </c>
     </row>
@@ -52033,7 +52113,7 @@
       </c>
       <c r="I331" s="7" t="inlineStr">
         <is>
-          <t>Evidence-tier reminder from the matrix figure applied while reviewing MD-00093. Logged as multimodal lead.</t>
+          <t>For MD-00093, multimodal policy figure is supporting context only (IT_asset_management_policy.pdf). Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -52209,7 +52289,7 @@
       </c>
       <c r="I335" s="7" t="inlineStr">
         <is>
-          <t>Assignment event TR-00094 on MD-00094 with APR-00094.</t>
+          <t>Receiving narrative for MD-00094 follows TR-00094 into Unknown.</t>
         </is>
       </c>
     </row>
@@ -52373,7 +52453,7 @@
       </c>
       <c r="I339" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00094; did not treat it as clearance. Returned to source files next.</t>
+          <t>Opened ITAM_control_matrix.png beside MD-00094; used as orientation, not clearance. Marked lead-only.</t>
         </is>
       </c>
     </row>
@@ -52549,7 +52629,7 @@
       </c>
       <c r="I343" s="7" t="inlineStr">
         <is>
-          <t>TR-00095 moved MD-00095; approval APR-00095.</t>
+          <t>Device MD-00095 hop evidenced solely by TR-00095.</t>
         </is>
       </c>
     </row>
@@ -52713,7 +52793,7 @@
       </c>
       <c r="I347" s="7" t="inlineStr">
         <is>
-          <t>Policy figure pass for MD-00095 completed before citing PO/TR/ticket identifiers. Logged as multimodal lead.</t>
+          <t>Reviewed control names on the PNG while documenting MD-00095; kept text records authoritative. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -52889,7 +52969,7 @@
       </c>
       <c r="I351" s="7" t="inlineStr">
         <is>
-          <t>MD-00096 changed hands under TR-00096; location context Unknown.</t>
+          <t>Assignment/transfer row TR-00096 kept as-is for MD-00096 [t351-1].</t>
         </is>
       </c>
     </row>
@@ -53053,7 +53133,7 @@
       </c>
       <c r="I355" s="7" t="inlineStr">
         <is>
-          <t>Opened ITAM_control_matrix.png next to MD-00096; used only to recall control expectations. Left as orientation.</t>
+          <t>ITAM matrix image used to confirm expected evidence classes for MD-00096. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -53229,7 +53309,7 @@
       </c>
       <c r="I359" s="7" t="inlineStr">
         <is>
-          <t>Assignment event TR-00097 on MD-00097 with APR-00097.</t>
+          <t>Record reference TR-00097 is the assignment spine for MD-00097.</t>
         </is>
       </c>
     </row>
@@ -53393,7 +53473,7 @@
       </c>
       <c r="I363" s="7" t="inlineStr">
         <is>
-          <t>Multimodal policy PNG referenced for MD-00097; text extracts remain authoritative. Marked lead-only.</t>
+          <t>For MD-00097, the policy figure clarifies evidence precedence without adding new facts. No clearance inferred.</t>
         </is>
       </c>
     </row>
@@ -53569,7 +53649,7 @@
       </c>
       <c r="I367" s="7" t="inlineStr">
         <is>
-          <t>TR-00098 moved MD-00098; approval APR-00098.</t>
+          <t>Transfer log TR-00098 governs the MD-00098 assignment event.</t>
         </is>
       </c>
     </row>
@@ -53733,7 +53813,7 @@
       </c>
       <c r="I371" s="7" t="inlineStr">
         <is>
-          <t>Control graphic for MD-00098 is informational; chain relies on register and transfer records. Did not elevate to proof.</t>
+          <t>ITAM_control_matrix.png cited once in the MD-00098 chain as a lead. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -53909,7 +53989,7 @@
       </c>
       <c r="I375" s="7" t="inlineStr">
         <is>
-          <t>MD-00099 changed hands under TR-00099; location context Unknown.</t>
+          <t>Hand-off documentation for MD-00099 = TR-00099 [t375-1].</t>
         </is>
       </c>
     </row>
@@ -54073,7 +54153,7 @@
       </c>
       <c r="I379" s="7" t="inlineStr">
         <is>
-          <t>Policy matrix figure reviewed for MD-00099 — assignment/return/disposal rows — then returned to source IDs. Marked lead-only.</t>
+          <t>Multimodal policy figure cited for MD-00099; text sources remain authoritative. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -54249,7 +54329,7 @@
       </c>
       <c r="I383" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00100 documented in TR-00100; site note Unknown.</t>
+          <t>Assignment evidence retained: TR-00100 for MD-00100.</t>
         </is>
       </c>
     </row>
@@ -54413,7 +54493,7 @@
       </c>
       <c r="I387" s="7" t="inlineStr">
         <is>
-          <t>Multimodal policy PNG referenced for MD-00100; text extracts remain authoritative. Did not elevate to proof.</t>
+          <t>No elevation of ITAM_control_matrix.png to clearance evidence for MD-00100. Marked lead-only.</t>
         </is>
       </c>
     </row>
@@ -54589,7 +54669,7 @@
       </c>
       <c r="I391" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00101 for MD-00101; receiving side Seattle.</t>
+          <t>Transfer TR-00101 listed against MD-00101 with site Seattle [t391-1].</t>
         </is>
       </c>
     </row>
@@ -54753,7 +54833,7 @@
       </c>
       <c r="I395" s="7" t="inlineStr">
         <is>
-          <t>Used ITAM_control_matrix.png as a checklist reminder for MD-00101, then verified against logs. No clearance inferred.</t>
+          <t>Control-matrix lead noted for MD-00101; evidence precedence still follows ITAM-001. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -54894,7 +54974,7 @@
       </c>
       <c r="I398" s="7" t="inlineStr">
         <is>
-          <t>MD-00102 changed hands under TR-00102; location context Atlanta.</t>
+          <t>Use source transfer TR-00102 when explaining MD-00102's move.</t>
         </is>
       </c>
     </row>
@@ -55058,7 +55138,7 @@
       </c>
       <c r="I402" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00102 working set; kept it marked as a lead. Marked lead-only.</t>
+          <t>Policy PNG pass on MD-00102 logged as multimodal lead under ITAM_control_matrix.png. Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -55199,7 +55279,7 @@
       </c>
       <c r="I405" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00103 for MD-00103; receiving side Chicago.</t>
+          <t>Custody movement for MD-00103 summarized from TR-00103 [t405-1].</t>
         </is>
       </c>
     </row>
@@ -55363,7 +55443,7 @@
       </c>
       <c r="I409" s="7" t="inlineStr">
         <is>
-          <t>Policy matrix figure reviewed for MD-00103 — assignment/return/disposal rows — then returned to source IDs. Returned to source files next.</t>
+          <t>Control matrix consulted; missing proof on MD-00103 still called out separately. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -55504,7 +55584,7 @@
       </c>
       <c r="I412" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00104 for MD-00104; receiving side Dallas.</t>
+          <t>TR-00104 remains the authoritative move record for MD-00104.</t>
         </is>
       </c>
     </row>
@@ -55668,7 +55748,7 @@
       </c>
       <c r="I416" s="7" t="inlineStr">
         <is>
-          <t>For MD-00104, the policy figure clarifies evidence precedence without adding new facts. Did not elevate to proof.</t>
+          <t>Evidence-tier reminder from the matrix figure applied while reviewing MD-00104. Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -55809,7 +55889,7 @@
       </c>
       <c r="I419" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00105 documented in TR-00105; site note Denver.</t>
+          <t>equipment_transfer_log TR-00105: custody hop for MD-00105.</t>
         </is>
       </c>
     </row>
@@ -55973,7 +56053,7 @@
       </c>
       <c r="I423" s="7" t="inlineStr">
         <is>
-          <t>ITAM PNG reviewed; MD-00105 still needs ordinary source documentation. Evidence tier reminder only.</t>
+          <t>Kept MD-00105 disposition independent of the policy figure visual. Did not elevate to proof.</t>
         </is>
       </c>
     </row>
@@ -56114,7 +56194,7 @@
       </c>
       <c r="I426" s="7" t="inlineStr">
         <is>
-          <t>MD-00106 changed hands under TR-00106; location context New York.</t>
+          <t>TR-00106 moved MD-00106; approval blank [t426-1].</t>
         </is>
       </c>
     </row>
@@ -56278,7 +56358,7 @@
       </c>
       <c r="I430" s="7" t="inlineStr">
         <is>
-          <t>Opened ITAM_control_matrix.png next to MD-00106; used only to recall control expectations. Returned to source files next.</t>
+          <t>Control PNG does not resolve open exceptions on MD-00106. No clearance inferred.</t>
         </is>
       </c>
     </row>
@@ -56419,7 +56499,7 @@
       </c>
       <c r="I433" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00107 relocates MD-00107 toward Seattle.</t>
+          <t>MD-00107 moved on TR-00107; no embellishment added.</t>
         </is>
       </c>
     </row>
@@ -56583,7 +56663,7 @@
       </c>
       <c r="I437" s="7" t="inlineStr">
         <is>
-          <t>Used ITAM_control_matrix.png as a checklist reminder for MD-00107, then verified against logs. Left as orientation.</t>
+          <t>ITAM matrix glance during MD-00107 chain build; disposition still needs PO/TR/ticket. Did not elevate to proof.</t>
         </is>
       </c>
     </row>
@@ -56724,7 +56804,7 @@
       </c>
       <c r="I440" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00108 for MD-00108; receiving side Atlanta.</t>
+          <t>equipment_transfer_log TR-00108: custody hop for MD-00108 [t440-1].</t>
         </is>
       </c>
     </row>
@@ -56888,7 +56968,7 @@
       </c>
       <c r="I444" s="7" t="inlineStr">
         <is>
-          <t>Matrix image confirms what proof is expected for MD-00108; it is not itself that proof. Logged as multimodal lead.</t>
+          <t>Figure review for MD-00108 finished before any disposition language was written. No clearance inferred.</t>
         </is>
       </c>
     </row>
@@ -57029,7 +57109,7 @@
       </c>
       <c r="I447" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00109 relocates MD-00109 toward Chicago.</t>
+          <t>Assignment event TR-00109 on MD-00109 without approval_id [t447-1].</t>
         </is>
       </c>
     </row>
@@ -57193,7 +57273,7 @@
       </c>
       <c r="I451" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00109 working set; kept it marked as a lead. No clearance inferred.</t>
+          <t>For MD-00109, the policy figure clarifies evidence precedence without adding new facts. Logged as multimodal lead.</t>
         </is>
       </c>
     </row>
@@ -57334,7 +57414,7 @@
       </c>
       <c r="I454" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00110 documented in TR-00110; site note Dallas.</t>
+          <t>Custody change on MD-00110 rests on transfer TR-00110.</t>
         </is>
       </c>
     </row>
@@ -57498,7 +57578,7 @@
       </c>
       <c r="I458" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00110 working set; kept it marked as a lead. Did not elevate to proof.</t>
+          <t>ITAM_control_matrix.png used as a checklist reminder for MD-00110, then verified against logs. Left as orientation.</t>
         </is>
       </c>
     </row>
@@ -57639,7 +57719,7 @@
       </c>
       <c r="I461" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00114 relocates MD-00114 toward Disposed.</t>
+          <t>Recorded relocation TR-00114 for MD-00114 into Disposed [t461-1].</t>
         </is>
       </c>
     </row>
@@ -57850,7 +57930,7 @@
       </c>
       <c r="I466" s="7" t="inlineStr">
         <is>
-          <t>Saw ITAM_control_matrix.png in the MD-00114 working set; kept it marked as a lead. Did not elevate to proof.</t>
+          <t>Multimodal lead logged for MD-00114 from ITAM_control_matrix.png without relying on it. Did not elevate to proof.</t>
         </is>
       </c>
     </row>
@@ -57991,7 +58071,7 @@
       </c>
       <c r="I469" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00118 documented in TR-00118; site note Disposed.</t>
+          <t>Use TR-00118 when reconstructing the MD-00118 custody hop [t469-1].</t>
         </is>
       </c>
     </row>
@@ -58202,7 +58282,7 @@
       </c>
       <c r="I474" s="7" t="inlineStr">
         <is>
-          <t>Multimodal policy PNG referenced for MD-00118; text extracts remain authoritative. Left as orientation.</t>
+          <t>For MD-00118, the policy figure clarifies evidence precedence without adding new facts. Did not elevate to proof.</t>
         </is>
       </c>
     </row>
@@ -58343,7 +58423,7 @@
       </c>
       <c r="I477" s="7" t="inlineStr">
         <is>
-          <t>MD-00119 changed hands under TR-00119; location context Disposed.</t>
+          <t>Chain event for MD-00119: transfer TR-00119 to Disposed [t477-1].</t>
         </is>
       </c>
     </row>
@@ -58554,7 +58634,7 @@
       </c>
       <c r="I482" s="7" t="inlineStr">
         <is>
-          <t>Used ITAM_control_matrix.png as a checklist reminder for MD-00119, then verified against logs. Marked lead-only.</t>
+          <t>Lead-only mark applied to the policy PNG entry for MD-00119. Returned to source files next [p482-1].</t>
         </is>
       </c>
     </row>
@@ -58687,7 +58767,7 @@
       </c>
       <c r="I485" s="7" t="inlineStr">
         <is>
-          <t>For MD-00127, the policy figure clarifies evidence precedence without adding new facts. Kept out of disposition logic.</t>
+          <t>Evidence-tier reminder from the matrix figure applied while reviewing MD-00127. Kept out of disposition logic.</t>
         </is>
       </c>
     </row>
@@ -58734,7 +58814,7 @@
       </c>
       <c r="I486" s="7" t="inlineStr">
         <is>
-          <t>Assignment event TR-00127 on MD-00127 without approval_id.</t>
+          <t>Move id TR-00127 anchors the assignment step for MD-00127 [t486-1].</t>
         </is>
       </c>
     </row>
@@ -58867,7 +58947,7 @@
       </c>
       <c r="I489" s="7" t="inlineStr">
         <is>
-          <t>Policy matrix figure reviewed for MD-00130 — assignment/return/disposal rows — then returned to source IDs. Returned to source files next.</t>
+          <t>ITAM_control_matrix.png remains a lead beside the MD-00130 chain. Evidence tier reminder only.</t>
         </is>
       </c>
     </row>
@@ -58914,7 +58994,7 @@
       </c>
       <c r="I490" s="7" t="inlineStr">
         <is>
-          <t>Hand-off for MD-00130 documented in TR-00130; site note Atlanta.</t>
+          <t>Custody hop language for MD-00130 mirrors TR-00130 fields [t490-1].</t>
         </is>
       </c>
     </row>
@@ -59055,7 +59135,7 @@
       </c>
       <c r="I493" s="7" t="inlineStr">
         <is>
-          <t>Logged transfer TR-00131 for MD-00131; receiving side Chicago.</t>
+          <t>Transfer proof on file for MD-00131: TR-00131.</t>
         </is>
       </c>
     </row>
@@ -59094,7 +59174,7 @@
       </c>
       <c r="I494" s="7" t="inlineStr">
         <is>
-          <t>Glanced at the control-matrix image while documenting MD-00131; did not treat it as clearance. No clearance inferred.</t>
+          <t>Policy figure pass for MD-00131 completed before citing PO/TR/ticket identifiers. Returned to source files next.</t>
         </is>
       </c>
     </row>
@@ -59235,7 +59315,7 @@
       </c>
       <c r="I497" s="7" t="inlineStr">
         <is>
-          <t>Transfer TR-00132 relocates MD-00132 toward Dallas.</t>
+          <t>MD-00132 reassigned under transfer TR-00132.</t>
         </is>
       </c>
     </row>
@@ -59274,7 +59354,7 @@
       </c>
       <c r="I498" s="7" t="inlineStr">
         <is>
-          <t>Used ITAM_control_matrix.png as a checklist reminder for MD-00132, then verified against logs. Did not elevate to proof.</t>
+          <t>Visual control checklist consulted for MD-00132; source IDs remain decisive. Returned to source files next [p498-1].</t>
         </is>
       </c>
     </row>
@@ -59399,6 +59479,304 @@
         </is>
       </c>
     </row>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -59441,6 +59819,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -59552,6 +59931,8 @@
         <v>3</v>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
@@ -59587,6 +59968,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
@@ -60044,6 +60426,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -60236,6 +60619,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
@@ -60395,6 +60779,7 @@
       <c r="D27" s="15" t="inlineStr"/>
       <c r="E27" s="15" t="inlineStr"/>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
@@ -60493,7 +60878,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EX-0092</t>
+          <t>OFF-00082; 1ZMD00000082; MISMATCH-0082</t>
         </is>
       </c>
     </row>
@@ -60625,6 +61010,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
         <is>

</xml_diff>